<commit_message>
v3: schedule risk (CPM), risk register, joint confidence, contingency split and allocation, web app
</commit_message>
<xml_diff>
--- a/data/sample_wbs.xlsx
+++ b/data/sample_wbs.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Matrix" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Matrix" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="£#,##0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +35,10 @@
     <font>
       <i val="1"/>
       <color rgb="00666666"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="0052514E"/>
     </font>
   </fonts>
   <fills count="4">
@@ -66,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -79,6 +84,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C2:K25"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -458,8 +473,14 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="C2" s="1" t="inlineStr">
         <is>
@@ -504,6 +525,31 @@
       <c r="K2" s="1" t="inlineStr">
         <is>
           <t>Risk % multiplier</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Duration (days)</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Optimistic Duration</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Pessimistic Duration</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Predecessors</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>Time-dependent %</t>
         </is>
       </c>
     </row>
@@ -572,6 +618,27 @@
       <c r="K4" t="n">
         <v>0.2</v>
       </c>
+      <c r="L4" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" s="11" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="5">
       <c r="C5" t="inlineStr">
@@ -609,6 +676,27 @@
       <c r="K5" t="n">
         <v>0.4</v>
       </c>
+      <c r="L5" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="P5" s="11" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="6">
       <c r="C6" t="inlineStr">
@@ -646,6 +734,27 @@
       <c r="K6" t="n">
         <v>0.6</v>
       </c>
+      <c r="L6" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="P6" s="11" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="7">
       <c r="C7" t="inlineStr">
@@ -683,6 +792,27 @@
       <c r="K7" t="n">
         <v>0.4</v>
       </c>
+      <c r="L7" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="P7" s="11" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
@@ -719,6 +849,27 @@
       </c>
       <c r="K8" t="n">
         <v>0.2</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>1.3, 1.2.1</t>
+        </is>
+      </c>
+      <c r="P8" s="11" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="9">
@@ -786,6 +937,27 @@
       <c r="K10" t="n">
         <v>0.4</v>
       </c>
+      <c r="L10" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="P10" s="11" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="C11" t="inlineStr">
@@ -823,6 +995,25 @@
       <c r="K11" t="n">
         <v>0.6</v>
       </c>
+      <c r="L11" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="P11" s="11" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="12">
       <c r="C12" t="inlineStr">
@@ -856,6 +1047,23 @@
       <c r="K12" t="n">
         <v>0.8</v>
       </c>
+      <c r="L12" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="M12" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="N12" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="P12" s="11" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="13">
       <c r="C13" t="inlineStr">
@@ -892,6 +1100,27 @@
       </c>
       <c r="K13" t="n">
         <v>0.2</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="P13" s="11" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="14">
@@ -959,6 +1188,27 @@
       <c r="K15" t="n">
         <v>0.4</v>
       </c>
+      <c r="L15" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N15" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O15" s="10" t="inlineStr">
+        <is>
+          <t>2.2, 2.3, 2.4</t>
+        </is>
+      </c>
+      <c r="P15" s="11" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
@@ -996,6 +1246,27 @@
       <c r="K16" t="n">
         <v>0.4</v>
       </c>
+      <c r="L16" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N16" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O16" s="10" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="P16" s="11" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="17">
       <c r="C17" t="inlineStr">
@@ -1033,6 +1304,27 @@
       <c r="K17" t="n">
         <v>0.4</v>
       </c>
+      <c r="L17" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="M17" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O17" s="10" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="P17" s="11" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="18">
       <c r="C18" t="inlineStr">
@@ -1069,6 +1361,25 @@
       </c>
       <c r="K18" t="n">
         <v>0.6</v>
+      </c>
+      <c r="L18" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="M18" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="O18" s="10" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="P18" s="11" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="19">
@@ -1136,6 +1447,27 @@
       <c r="K20" t="n">
         <v>0.2</v>
       </c>
+      <c r="L20" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="P20" s="11" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">
@@ -1173,6 +1505,27 @@
       <c r="K21" t="n">
         <v>0.6</v>
       </c>
+      <c r="L21" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="M21" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N21" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>4.1, 3.3.1</t>
+        </is>
+      </c>
+      <c r="P21" s="11" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="22">
       <c r="C22" t="inlineStr">
@@ -1210,6 +1563,27 @@
       <c r="K22" t="n">
         <v>0.2</v>
       </c>
+      <c r="L22" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="M22" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N22" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="10" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="P22" s="11" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="23">
       <c r="C23" t="inlineStr">
@@ -1242,6 +1616,23 @@
       </c>
       <c r="K23" t="n">
         <v>0.2</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="N23" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>4.2, 4.3</t>
+        </is>
+      </c>
+      <c r="P23" s="11" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="24"/>
@@ -1258,6 +1649,351 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Risk register: each risk either happens (by its probability) or not. Cost impacts are added to the total; schedule impacts extend the affected task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Risk ID</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Probability (%)</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Cost impact min</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Cost impact most likely</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Cost impact max</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Schedule impact min (days)</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Schedule impact most likely (days)</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Schedule impact max (days)</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Affected task</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Integration vendor delivers its API late</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Technical lead</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Legacy data quality worse than the audit suggested</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Data lead</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>50</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" t="n">
+        <v>15</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Key business experts unavailable during UAT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Business sponsor</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Security testing finds a critical vulnerability</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Security lead</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10</v>
+      </c>
+      <c r="J7" t="n">
+        <v>20</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Regulator requests a scope change mid-build</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Project manager</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" t="n">
+        <v>30</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Software licence price rises at renewal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Commercial lead</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>35</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>